<commit_message>
Update SQS logic and improve Python script robustness
- Switches SQS agent and global average calculation to Simple Average instead of Weighted Average per user rule.
- Updates both `gerar_hitlist.py` and `macro_vba.txt` for this rule.
- Modifies Python script to handle case insensitive dates, resolve division by zero warnings for 100% ABS agents, use outer joins, and dynamically fetch the Answered column name based on index.
</commit_message>
<xml_diff>
--- a/TO Hitlist.xlsx
+++ b/TO Hitlist.xlsx
@@ -5038,7 +5038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5058,7 +5058,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>% SQS Global: 87.52%</t>
+          <t>% SQS Global: 88.35%</t>
         </is>
       </c>
     </row>
@@ -5159,13 +5159,13 @@
         </is>
       </c>
       <c r="G8" s="14" t="n">
-        <v>0.7678571492433548</v>
+        <v>0.8076190527280172</v>
       </c>
       <c r="H8" s="14" t="n">
         <v>16</v>
       </c>
       <c r="I8" s="14" t="n">
-        <v>-1.717902331412594</v>
+        <v>-1.213726364317393</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -5179,31 +5179,31 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MARIA JOSE</t>
+          <t>VICTOR</t>
         </is>
       </c>
       <c r="B9" s="14" t="n">
-        <v>0.8709677419354839</v>
+        <v>0</v>
       </c>
       <c r="C9" s="14" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>0.4819277108433743</v>
+        <v>-0</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ZEMA</t>
+          <t>VICTOR</t>
         </is>
       </c>
       <c r="G9" s="14" t="n">
-        <v>0.8775510266423225</v>
+        <v>0</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="I9" s="14" t="n">
-        <v>0.06509948719905756</v>
+        <v>-0</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -5217,31 +5217,31 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>JOSE MARIA</t>
+          <t>MARIA JOSE</t>
         </is>
       </c>
       <c r="B10" s="14" t="n">
-        <v>0.875</v>
+        <v>0.8709677419354839</v>
       </c>
       <c r="C10" s="14" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>0.6265060240963862</v>
+        <v>0.4819277108433743</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>MARIA JOSE</t>
+          <t>ZEMA</t>
         </is>
       </c>
       <c r="G10" s="14" t="n">
-        <v>0.9224489833627428</v>
+        <v>0.9088435418549038</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="I10" s="14" t="n">
-        <v>1.652802844213532</v>
+        <v>0.7102645579973874</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -5252,7 +5252,44 @@
         <v>0.3894820804195804</v>
       </c>
     </row>
-    <row r="11"/>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>JOSE MARIA</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>32</v>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>0.6265060240963862</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>MARIA JOSE</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>0.9339682569106419</v>
+      </c>
+      <c r="H11" s="14" t="n">
+        <v>35</v>
+      </c>
+      <c r="I11" s="14" t="n">
+        <v>1.767195724447568</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>VICTOR</t>
+        </is>
+      </c>
+      <c r="L11" s="14" t="n">
+        <v>0.3138888888888889</v>
+      </c>
+    </row>
     <row r="12"/>
     <row r="13"/>
     <row r="14"/>
@@ -5365,10 +5402,10 @@
         <v>0.6265060240963862</v>
       </c>
       <c r="C22" s="14" t="n">
-        <v>-1.717902331412594</v>
+        <v>-1.213726364317393</v>
       </c>
       <c r="D22" s="14" t="n">
-        <v>-1.091396307316208</v>
+        <v>-0.5872203402210072</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -5376,7 +5413,7 @@
         </is>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-1.091396307316208</v>
+        <v>-0.5872203402210072</v>
       </c>
       <c r="H22" s="14" t="n">
         <v>0.6169780643738977</v>
@@ -5390,10 +5427,10 @@
         <v>1.553907668287096</v>
       </c>
       <c r="L22" s="14" t="n">
-        <v>-4.260871409816836</v>
+        <v>-3.010376009448963</v>
       </c>
       <c r="M22" s="14" t="n">
-        <v>-2.70696374152974</v>
+        <v>-1.456468341161867</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -5401,7 +5438,7 @@
         </is>
       </c>
       <c r="P22" s="14" t="n">
-        <v>-2.70696374152974</v>
+        <v>-1.456468341161867</v>
       </c>
       <c r="Q22" s="14" t="n">
         <v>0.6169780643738977</v>
@@ -5417,10 +5454,10 @@
         <v>-1.108433734939758</v>
       </c>
       <c r="C23" s="14" t="n">
-        <v>0.06509948719905756</v>
+        <v>0.7102645579973874</v>
       </c>
       <c r="D23" s="14" t="n">
-        <v>-1.0433342477407</v>
+        <v>-0.3981691769423703</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -5428,7 +5465,7 @@
         </is>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-1.0433342477407</v>
+        <v>-0.3981691769423703</v>
       </c>
       <c r="H23" s="14" t="n">
         <v>0.3894820804195804</v>
@@ -5442,10 +5479,10 @@
         <v>-1.724784833369766</v>
       </c>
       <c r="L23" s="14" t="n">
-        <v>0.09299926742722509</v>
+        <v>1.014663654281982</v>
       </c>
       <c r="M23" s="14" t="n">
-        <v>-1.63178556594254</v>
+        <v>-0.7101211790877835</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -5453,7 +5490,7 @@
         </is>
       </c>
       <c r="P23" s="14" t="n">
-        <v>-1.63178556594254</v>
+        <v>-0.7101211790877835</v>
       </c>
       <c r="Q23" s="14" t="n">
         <v>0.3894820804195804</v>
@@ -5462,52 +5499,104 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>VICTOR</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="n">
+        <v>-0</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D24" s="14" t="n">
+        <v>-0</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>VICTOR</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>0.3138888888888889</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>VICTOR</t>
+        </is>
+      </c>
+      <c r="K24" s="14" t="n">
+        <v>-0</v>
+      </c>
+      <c r="L24" s="14" t="n">
+        <v>-0</v>
+      </c>
+      <c r="M24" s="14" t="n">
+        <v>-0</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>VICTOR</t>
+        </is>
+      </c>
+      <c r="P24" s="14" t="n">
+        <v>-0</v>
+      </c>
+      <c r="Q24" s="14" t="n">
+        <v>0.3138888888888889</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>MARIA JOSE</t>
         </is>
       </c>
-      <c r="B24" s="14" t="n">
+      <c r="B25" s="14" t="n">
         <v>0.4819277108433743</v>
       </c>
-      <c r="C24" s="14" t="n">
-        <v>1.652802844213532</v>
-      </c>
-      <c r="D24" s="14" t="n">
-        <v>2.134730555056906</v>
-      </c>
-      <c r="F24" t="inlineStr">
+      <c r="C25" s="14" t="n">
+        <v>1.767195724447568</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>2.249123435290942</v>
+      </c>
+      <c r="F25" t="inlineStr">
         <is>
           <t>MARIA JOSE</t>
         </is>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>2.134730555056906</v>
-      </c>
-      <c r="H24" s="14" t="n">
+      <c r="G25" s="14" t="n">
+        <v>2.249123435290942</v>
+      </c>
+      <c r="H25" s="14" t="n">
         <v>0.4910774410774411</v>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>MARIA JOSE</t>
         </is>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="K25" s="14" t="n">
         <v>0.8996090215974731</v>
       </c>
-      <c r="L24" s="14" t="n">
-        <v>1.888917536244037</v>
-      </c>
-      <c r="M24" s="14" t="n">
-        <v>2.78852655784151</v>
-      </c>
-      <c r="O24" t="inlineStr">
+      <c r="L25" s="14" t="n">
+        <v>2.019652256511506</v>
+      </c>
+      <c r="M25" s="14" t="n">
+        <v>2.919261278108979</v>
+      </c>
+      <c r="O25" t="inlineStr">
         <is>
           <t>MARIA JOSE</t>
         </is>
       </c>
-      <c r="P24" s="14" t="n">
-        <v>2.78852655784151</v>
-      </c>
-      <c r="Q24" s="14" t="n">
+      <c r="P25" s="14" t="n">
+        <v>2.919261278108979</v>
+      </c>
+      <c r="Q25" s="14" t="n">
         <v>0.4910774410774411</v>
       </c>
     </row>

</xml_diff>